<commit_message>
feat: dispatch 175 deep research leads, conduct IMAP deliverability audit, and update omnichannel Excel tracker
</commit_message>
<xml_diff>
--- a/data/MASTER_CRM_OPERATIONS.xlsx
+++ b/data/MASTER_CRM_OPERATIONS.xlsx
@@ -273,7 +273,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -400,7 +400,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA39" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA40" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA41" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA42" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA43" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA46" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA47" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA48" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA49" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA50" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA51" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="Z55" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA55" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="Z56" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA56" t="inlineStr">
@@ -7258,7 +7258,7 @@
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA57" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -7512,7 +7512,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
@@ -7639,7 +7639,7 @@
       </c>
       <c r="Z60" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA60" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA61" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA62" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="Z63" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA63" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA64" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="Z65" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA65" t="inlineStr">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="Z67" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA67" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="Z68" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA68" t="inlineStr">
@@ -8782,7 +8782,7 @@
       </c>
       <c r="Z69" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA69" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="Z70" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA70" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="Z71" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA71" t="inlineStr">
@@ -9163,7 +9163,7 @@
       </c>
       <c r="Z72" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA72" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="Z73" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA73" t="inlineStr">
@@ -9417,7 +9417,7 @@
       </c>
       <c r="Z74" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA74" t="inlineStr">
@@ -9544,7 +9544,7 @@
       </c>
       <c r="Z75" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA75" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA76" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="Z77" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA77" t="inlineStr">
@@ -9925,7 +9925,7 @@
       </c>
       <c r="Z78" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA78" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="Z79" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA79" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="Z80" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA80" t="inlineStr">
@@ -10306,7 +10306,7 @@
       </c>
       <c r="Z81" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA81" t="inlineStr">
@@ -10433,7 +10433,7 @@
       </c>
       <c r="Z82" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA82" t="inlineStr">
@@ -10560,7 +10560,7 @@
       </c>
       <c r="Z83" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA83" t="inlineStr">
@@ -10687,7 +10687,7 @@
       </c>
       <c r="Z84" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA84" t="inlineStr">
@@ -10814,7 +10814,7 @@
       </c>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA85" t="inlineStr">
@@ -10941,7 +10941,7 @@
       </c>
       <c r="Z86" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA86" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="Z87" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA87" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="Z88" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA88" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="Z89" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA89" t="inlineStr">
@@ -11449,7 +11449,7 @@
       </c>
       <c r="Z90" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA90" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="Z91" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA91" t="inlineStr">
@@ -11703,7 +11703,7 @@
       </c>
       <c r="Z92" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA92" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="Z93" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA93" t="inlineStr">
@@ -11957,7 +11957,7 @@
       </c>
       <c r="Z94" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA94" t="inlineStr">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="Z95" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA95" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="Z96" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA96" t="inlineStr">
@@ -12338,7 +12338,7 @@
       </c>
       <c r="Z97" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA97" t="inlineStr">
@@ -12465,7 +12465,7 @@
       </c>
       <c r="Z98" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA98" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="Z99" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA99" t="inlineStr">
@@ -12719,7 +12719,7 @@
       </c>
       <c r="Z100" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA100" t="inlineStr">
@@ -12846,7 +12846,7 @@
       </c>
       <c r="Z101" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA101" t="inlineStr">
@@ -12973,7 +12973,7 @@
       </c>
       <c r="Z102" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA102" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="Z103" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA103" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="Z104" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA104" t="inlineStr">
@@ -13354,7 +13354,7 @@
       </c>
       <c r="Z105" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA105" t="inlineStr">
@@ -13481,7 +13481,7 @@
       </c>
       <c r="Z106" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA106" t="inlineStr">
@@ -13608,7 +13608,7 @@
       </c>
       <c r="Z107" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA107" t="inlineStr">
@@ -13735,7 +13735,7 @@
       </c>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA108" t="inlineStr">
@@ -13862,7 +13862,7 @@
       </c>
       <c r="Z109" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA109" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="Z110" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA110" t="inlineStr">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA111" t="inlineStr">
@@ -14243,7 +14243,7 @@
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA112" t="inlineStr">
@@ -14370,7 +14370,7 @@
       </c>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA113" t="inlineStr">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="Z114" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA114" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="Z115" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA115" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="Z116" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA116" t="inlineStr">
@@ -14878,7 +14878,7 @@
       </c>
       <c r="Z117" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA117" t="inlineStr">
@@ -15005,7 +15005,7 @@
       </c>
       <c r="Z118" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA118" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="Z119" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA119" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="Z120" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA120" t="inlineStr">
@@ -15386,7 +15386,7 @@
       </c>
       <c r="Z121" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA121" t="inlineStr">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="Z122" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA122" t="inlineStr">
@@ -15640,7 +15640,7 @@
       </c>
       <c r="Z123" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA123" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="Z124" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA124" t="inlineStr">
@@ -15894,7 +15894,7 @@
       </c>
       <c r="Z125" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA125" t="inlineStr">
@@ -16021,7 +16021,7 @@
       </c>
       <c r="Z126" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA126" t="inlineStr">
@@ -16148,7 +16148,7 @@
       </c>
       <c r="Z127" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA127" t="inlineStr">
@@ -16275,7 +16275,7 @@
       </c>
       <c r="Z128" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA128" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="Z129" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA129" t="inlineStr">
@@ -16529,7 +16529,7 @@
       </c>
       <c r="Z130" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA130" t="inlineStr">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="Z131" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA131" t="inlineStr">
@@ -16783,7 +16783,7 @@
       </c>
       <c r="Z132" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA132" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="Z133" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA133" t="inlineStr">
@@ -17037,7 +17037,7 @@
       </c>
       <c r="Z134" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA134" t="inlineStr">
@@ -17164,7 +17164,7 @@
       </c>
       <c r="Z135" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA135" t="inlineStr">
@@ -17291,7 +17291,7 @@
       </c>
       <c r="Z136" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA136" t="inlineStr">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="Z137" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA137" t="inlineStr">
@@ -17545,7 +17545,7 @@
       </c>
       <c r="Z138" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA138" t="inlineStr">
@@ -17672,7 +17672,7 @@
       </c>
       <c r="Z139" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA139" t="inlineStr">
@@ -17799,7 +17799,7 @@
       </c>
       <c r="Z140" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA140" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="Z141" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA141" t="inlineStr">
@@ -18053,7 +18053,7 @@
       </c>
       <c r="Z142" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA142" t="inlineStr">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="Z143" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA143" t="inlineStr">
@@ -18307,7 +18307,7 @@
       </c>
       <c r="Z144" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA144" t="inlineStr">
@@ -18434,7 +18434,7 @@
       </c>
       <c r="Z145" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA145" t="inlineStr">
@@ -18561,7 +18561,7 @@
       </c>
       <c r="Z146" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA146" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="Z147" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA147" t="inlineStr">
@@ -18815,7 +18815,7 @@
       </c>
       <c r="Z148" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA148" t="inlineStr">
@@ -18942,7 +18942,7 @@
       </c>
       <c r="Z149" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA149" t="inlineStr">
@@ -19069,7 +19069,7 @@
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr">
@@ -19196,7 +19196,7 @@
       </c>
       <c r="Z151" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA151" t="inlineStr">
@@ -19323,7 +19323,7 @@
       </c>
       <c r="Z152" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA152" t="inlineStr">
@@ -19450,7 +19450,7 @@
       </c>
       <c r="Z153" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA153" t="inlineStr">
@@ -19577,7 +19577,7 @@
       </c>
       <c r="Z154" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA154" t="inlineStr">
@@ -19704,7 +19704,7 @@
       </c>
       <c r="Z155" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA155" t="inlineStr">
@@ -19831,7 +19831,7 @@
       </c>
       <c r="Z156" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA156" t="inlineStr">
@@ -19958,7 +19958,7 @@
       </c>
       <c r="Z157" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA157" t="inlineStr">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="Z158" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA158" t="inlineStr">
@@ -20212,7 +20212,7 @@
       </c>
       <c r="Z159" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA159" t="inlineStr">
@@ -20339,7 +20339,7 @@
       </c>
       <c r="Z160" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA160" t="inlineStr">
@@ -20466,7 +20466,7 @@
       </c>
       <c r="Z161" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA161" t="inlineStr">
@@ -20593,7 +20593,7 @@
       </c>
       <c r="Z162" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA162" t="inlineStr">
@@ -20720,7 +20720,7 @@
       </c>
       <c r="Z163" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA163" t="inlineStr">
@@ -20847,7 +20847,7 @@
       </c>
       <c r="Z164" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA164" t="inlineStr">
@@ -20974,7 +20974,7 @@
       </c>
       <c r="Z165" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA165" t="inlineStr">
@@ -21101,7 +21101,7 @@
       </c>
       <c r="Z166" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA166" t="inlineStr">
@@ -21228,7 +21228,7 @@
       </c>
       <c r="Z167" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA167" t="inlineStr">
@@ -21355,7 +21355,7 @@
       </c>
       <c r="Z168" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA168" t="inlineStr">
@@ -21482,7 +21482,7 @@
       </c>
       <c r="Z169" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA169" t="inlineStr">
@@ -21609,7 +21609,7 @@
       </c>
       <c r="Z170" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA170" t="inlineStr">
@@ -21736,7 +21736,7 @@
       </c>
       <c r="Z171" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA171" t="inlineStr">
@@ -21863,7 +21863,7 @@
       </c>
       <c r="Z172" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA172" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="Z173" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA173" t="inlineStr">
@@ -22117,7 +22117,7 @@
       </c>
       <c r="Z174" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA174" t="inlineStr">
@@ -22244,7 +22244,7 @@
       </c>
       <c r="Z175" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA175" t="inlineStr">
@@ -22371,7 +22371,7 @@
       </c>
       <c r="Z176" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA176" t="inlineStr">
@@ -22498,7 +22498,7 @@
       </c>
       <c r="Z177" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA177" t="inlineStr">
@@ -22625,7 +22625,7 @@
       </c>
       <c r="Z178" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA178" t="inlineStr">
@@ -22752,7 +22752,7 @@
       </c>
       <c r="Z179" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA179" t="inlineStr">
@@ -22879,7 +22879,7 @@
       </c>
       <c r="Z180" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA180" t="inlineStr">
@@ -23006,7 +23006,7 @@
       </c>
       <c r="Z181" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA181" t="inlineStr">
@@ -23133,7 +23133,7 @@
       </c>
       <c r="Z182" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA182" t="inlineStr">
@@ -23260,7 +23260,7 @@
       </c>
       <c r="Z183" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA183" t="inlineStr">
@@ -23387,7 +23387,7 @@
       </c>
       <c r="Z184" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA184" t="inlineStr">
@@ -23514,7 +23514,7 @@
       </c>
       <c r="Z185" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA185" t="inlineStr">
@@ -23641,7 +23641,7 @@
       </c>
       <c r="Z186" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA186" t="inlineStr">
@@ -23768,7 +23768,7 @@
       </c>
       <c r="Z187" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA187" t="inlineStr">
@@ -23895,7 +23895,7 @@
       </c>
       <c r="Z188" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA188" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="Z189" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA189" t="inlineStr">
@@ -24149,7 +24149,7 @@
       </c>
       <c r="Z190" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA190" t="inlineStr">
@@ -24276,7 +24276,7 @@
       </c>
       <c r="Z191" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA191" t="inlineStr">
@@ -24403,7 +24403,7 @@
       </c>
       <c r="Z192" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA192" t="inlineStr">
@@ -24530,7 +24530,7 @@
       </c>
       <c r="Z193" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA193" t="inlineStr">
@@ -24657,7 +24657,7 @@
       </c>
       <c r="Z194" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA194" t="inlineStr">
@@ -24784,7 +24784,7 @@
       </c>
       <c r="Z195" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA195" t="inlineStr">
@@ -24911,7 +24911,7 @@
       </c>
       <c r="Z196" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA196" t="inlineStr">
@@ -25038,7 +25038,7 @@
       </c>
       <c r="Z197" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA197" t="inlineStr">
@@ -25165,7 +25165,7 @@
       </c>
       <c r="Z198" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA198" t="inlineStr">
@@ -25292,7 +25292,7 @@
       </c>
       <c r="Z199" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA199" t="inlineStr">
@@ -25419,7 +25419,7 @@
       </c>
       <c r="Z200" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA200" t="inlineStr">
@@ -25546,7 +25546,7 @@
       </c>
       <c r="Z201" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA201" t="inlineStr">
@@ -25673,7 +25673,7 @@
       </c>
       <c r="Z202" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA202" t="inlineStr">
@@ -25800,7 +25800,7 @@
       </c>
       <c r="Z203" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA203" t="inlineStr">
@@ -26071,7 +26071,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -26198,7 +26198,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -26325,7 +26325,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -26452,7 +26452,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -26579,7 +26579,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -26833,7 +26833,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -26960,7 +26960,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -27087,7 +27087,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>2026-09-04 21:28:33 UTC</t>
+          <t>2026-09-04 21:55:05 UTC</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">

</xml_diff>